<commit_message>
Configure GitHub Actions CI/CD to run all 4 E2E/Load/Security tests and upload Excel reports as artifacts
</commit_message>
<xml_diff>
--- a/QA_Reports/load_test_report.xlsx
+++ b/QA_Reports/load_test_report.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>4021 ms</t>
+          <t>4022 ms</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>4047 ms</t>
+          <t>4054 ms</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>4107 ms</t>
+          <t>4104 ms</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">

</xml_diff>